<commit_message>
Added .toml file to customize streamlit
</commit_message>
<xml_diff>
--- a/data/Budget2026.xlsx
+++ b/data/Budget2026.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="Departments"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="48">
   <si>
     <t>Expense_ID</t>
   </si>
@@ -30,18 +30,96 @@
     <t>amount</t>
   </si>
   <si>
-    <t>Software</t>
+    <t>Cloud Infrastructure</t>
+  </si>
+  <si>
+    <t>Cybersecurity</t>
+  </si>
+  <si>
+    <t>Software Licensing</t>
   </si>
   <si>
     <t>Hardware</t>
   </si>
   <si>
+    <t>AI Services</t>
+  </si>
+  <si>
+    <t>Digital Marketing</t>
+  </si>
+  <si>
     <t>Advertising</t>
   </si>
   <si>
+    <t>Events</t>
+  </si>
+  <si>
+    <t>Recruiting</t>
+  </si>
+  <si>
     <t>Training</t>
   </si>
   <si>
+    <t>Benefits</t>
+  </si>
+  <si>
+    <t>Audit</t>
+  </si>
+  <si>
+    <t>Consulting</t>
+  </si>
+  <si>
+    <t>Banking Fees</t>
+  </si>
+  <si>
+    <t>Sales Commissions</t>
+  </si>
+  <si>
+    <t>Travel</t>
+  </si>
+  <si>
+    <t>CRM Software</t>
+  </si>
+  <si>
+    <t>Equipment</t>
+  </si>
+  <si>
+    <t>Fleet</t>
+  </si>
+  <si>
+    <t>Utilities</t>
+  </si>
+  <si>
+    <t>Call Center</t>
+  </si>
+  <si>
+    <t>Help Desk Software</t>
+  </si>
+  <si>
+    <t>Lab Equipment</t>
+  </si>
+  <si>
+    <t>Prototypes</t>
+  </si>
+  <si>
+    <t>Outside Counsel</t>
+  </si>
+  <si>
+    <t>Compliance</t>
+  </si>
+  <si>
+    <t>Building Maintenance</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>Cleaning Services</t>
+  </si>
+  <si>
+    <t>Networking</t>
+  </si>
+  <si>
     <t>Budget_ID</t>
   </si>
   <si>
@@ -64,6 +142,24 @@
   </si>
   <si>
     <t>Finance</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>Operations</t>
+  </si>
+  <si>
+    <t>Customer Support</t>
+  </si>
+  <si>
+    <t>Research</t>
+  </si>
+  <si>
+    <t>Legal</t>
+  </si>
+  <si>
+    <t>Facilities</t>
   </si>
 </sst>
 </file>
@@ -106,12 +202,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFc6c6c6"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFc6c6c6"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFc6c6c6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -172,13 +283,13 @@
   </cellStyleXfs>
   <cellXfs count="11">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -190,16 +301,16 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="5" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -504,7 +615,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="5" width="13.147857142857141" customWidth="1" bestFit="1"/>
@@ -516,39 +627,87 @@
         <v>1</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
       <c r="A2" s="3">
-        <v>1</v>
+        <v>101</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
       <c r="A3" s="3">
-        <v>2</v>
+        <v>102</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
       <c r="A4" s="3">
-        <v>3</v>
+        <v>103</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
       <c r="A5" s="3">
-        <v>4</v>
+        <v>104</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>15</v>
+        <v>41</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
+      <c r="A6" s="3">
+        <v>105</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
+      <c r="A7" s="3">
+        <v>106</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
+      <c r="A8" s="3">
+        <v>107</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
+      <c r="A9" s="3">
+        <v>108</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
+      <c r="A10" s="3">
+        <v>109</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
+      <c r="A11" s="3">
+        <v>110</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -561,84 +720,180 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="5" width="13.147857142857141" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="5" width="16.576428571428572" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="16.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
       <c r="A1" s="7" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>10</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="E1" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
       <c r="B2" s="3">
-        <v>1</v>
+        <v>101</v>
       </c>
       <c r="C2" s="3">
         <v>2026</v>
       </c>
       <c r="D2" s="3">
-        <v>10000000</v>
-      </c>
+        <v>5800000</v>
+      </c>
+      <c r="E2" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" s="3">
-        <v>2</v>
+        <v>102</v>
       </c>
       <c r="C3" s="3">
         <v>2026</v>
       </c>
       <c r="D3" s="3">
-        <v>12000000</v>
-      </c>
+        <v>4200000</v>
+      </c>
+      <c r="E3" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
       <c r="B4" s="3">
-        <v>3</v>
+        <v>103</v>
       </c>
       <c r="C4" s="3">
         <v>2026</v>
       </c>
       <c r="D4" s="3">
-        <v>20000000</v>
-      </c>
+        <v>3200000</v>
+      </c>
+      <c r="E4" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
       <c r="B5" s="3">
-        <v>4</v>
+        <v>104</v>
       </c>
       <c r="C5" s="3">
         <v>2026</v>
       </c>
       <c r="D5" s="3">
-        <v>7000000</v>
-      </c>
+        <v>4700000</v>
+      </c>
+      <c r="E5" s="4"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3">
+        <v>105</v>
+      </c>
+      <c r="C6" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D6" s="3">
+        <v>9800000</v>
+      </c>
+      <c r="E6" s="4"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3">
+        <v>106</v>
+      </c>
+      <c r="C7" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D7" s="3">
+        <v>15500000</v>
+      </c>
+      <c r="E7" s="4"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3">
+        <v>107</v>
+      </c>
+      <c r="C8" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D8" s="3">
+        <v>5400000</v>
+      </c>
+      <c r="E8" s="4"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3">
+        <v>108</v>
+      </c>
+      <c r="C9" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D9" s="3">
+        <v>8700000</v>
+      </c>
+      <c r="E9" s="4"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3">
+        <v>109</v>
+      </c>
+      <c r="C10" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D10" s="3">
+        <v>2600000</v>
+      </c>
+      <c r="E10" s="4"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3">
+        <v>110</v>
+      </c>
+      <c r="C11" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D11" s="3">
+        <v>3900000</v>
+      </c>
+      <c r="E11" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -650,16 +905,16 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="5" width="10.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="13.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="10.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="6" width="18.862142857142857" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="5" width="7.576428571428571" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -678,13 +933,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="3">
-        <v>1</v>
+        <v>101</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>4</v>
       </c>
       <c r="D2" s="3">
-        <v>5000</v>
+        <v>127500</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
@@ -692,13 +947,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="3">
-        <v>1</v>
+        <v>101</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>5</v>
       </c>
       <c r="D3" s="3">
-        <v>12000</v>
+        <v>84500</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
@@ -706,13 +961,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="3">
-        <v>2</v>
+        <v>101</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="3">
-        <v>7000</v>
+        <v>39200</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
@@ -720,13 +975,377 @@
         <v>4</v>
       </c>
       <c r="B5" s="3">
-        <v>3</v>
+        <v>101</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="3">
-        <v>5000</v>
+        <v>112300</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3">
+        <v>101</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="3">
+        <v>18400</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3">
+        <v>102</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="3">
+        <v>236000</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3">
+        <v>102</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="3">
+        <v>174500</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3">
+        <v>102</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="3">
+        <v>68500</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3">
+        <v>103</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="3">
+        <v>41200</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3">
+        <v>103</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="3">
+        <v>18600</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="17.25">
+      <c r="A12" s="3">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3">
+        <v>103</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="3">
+        <v>318400</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25">
+      <c r="A13" s="3">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3">
+        <v>104</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" s="3">
+        <v>92700</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
+      <c r="A14" s="3">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3">
+        <v>104</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" s="3">
+        <v>146800</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
+      <c r="A15" s="3">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3">
+        <v>104</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D15" s="3">
+        <v>12400</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
+      <c r="A16" s="3">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3">
+        <v>105</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="3">
+        <v>452300</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25">
+      <c r="A17" s="3">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3">
+        <v>105</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" s="3">
+        <v>58300</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25">
+      <c r="A18" s="3">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3">
+        <v>105</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" s="3">
+        <v>94700</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
+      <c r="A19" s="3">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3">
+        <v>106</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D19" s="3">
+        <v>385000</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25">
+      <c r="A20" s="3">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3">
+        <v>106</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" s="3">
+        <v>214500</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="17.25">
+      <c r="A21" s="3">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3">
+        <v>106</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21" s="3">
+        <v>72600</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="17.25">
+      <c r="A22" s="3">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3">
+        <v>107</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" s="3">
+        <v>68900</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="17.25">
+      <c r="A23" s="3">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3">
+        <v>107</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D23" s="3">
+        <v>28400</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="17.25">
+      <c r="A24" s="3">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3">
+        <v>108</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D24" s="3">
+        <v>226000</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="17.25">
+      <c r="A25" s="3">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3">
+        <v>108</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D25" s="3">
+        <v>135400</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="17.25">
+      <c r="A26" s="3">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3">
+        <v>109</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D26" s="3">
+        <v>128700</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="17.25">
+      <c r="A27" s="3">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3">
+        <v>109</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D27" s="3">
+        <v>39200</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="17.25">
+      <c r="A28" s="3">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3">
+        <v>110</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D28" s="3">
+        <v>117800</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="17.25">
+      <c r="A29" s="3">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3">
+        <v>110</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D29" s="3">
+        <v>98500</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="17.25">
+      <c r="A30" s="3">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3">
+        <v>110</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D30" s="3">
+        <v>46300</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="17.25">
+      <c r="A31" s="3">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3">
+        <v>101</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D31" s="3">
+        <v>156900</v>
       </c>
     </row>
   </sheetData>

</xml_diff>